<commit_message>
feat(proto): 添加 proto 消息模板
</commit_message>
<xml_diff>
--- a/assets/xls/物品.xlsx
+++ b/assets/xls/物品.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="167">
   <si>
     <t>ID</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>cs</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
   <si>
     <t>编号</t>
@@ -1176,14 +1182,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1567,92 +1570,92 @@
     <col min="7" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="1" spans="1:6">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="1" spans="1:6">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" s="6" customFormat="1" spans="1:6">
-      <c r="A2" s="6" t="s">
+    <row r="2" s="5" customFormat="1" spans="1:6">
+      <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" s="6" customFormat="1" spans="1:6">
-      <c r="A3" s="6" t="s">
+    <row r="3" s="5" customFormat="1" spans="1:6">
+      <c r="A3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" s="6" customFormat="1" spans="1:6">
-      <c r="A4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="6" t="s">
+    </row>
+    <row r="4" s="5" customFormat="1" spans="1:6">
+      <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" s="6" customFormat="1" spans="1:6">
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" s="5" customFormat="1" spans="1:6">
       <c r="A5" s="1">
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1">
         <v>1</v>
@@ -1661,7 +1664,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="1"/>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <v>10</v>
       </c>
     </row>
@@ -1670,7 +1673,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
@@ -1679,7 +1682,7 @@
         <v>2</v>
       </c>
       <c r="E6" s="1"/>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <v>1000</v>
       </c>
     </row>
@@ -1688,7 +1691,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
@@ -1697,7 +1700,7 @@
         <v>3</v>
       </c>
       <c r="E7" s="1"/>
-      <c r="F7" s="7">
+      <c r="F7" s="6">
         <v>10000</v>
       </c>
     </row>
@@ -1706,7 +1709,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" s="1">
         <v>2</v>
@@ -1714,7 +1717,7 @@
       <c r="D8" s="1">
         <v>4</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="6">
         <v>100000000</v>
       </c>
     </row>
@@ -1723,7 +1726,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C9" s="1">
         <v>888</v>
@@ -1731,7 +1734,7 @@
       <c r="D9" s="1">
         <v>5</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="6">
         <v>999999999</v>
       </c>
     </row>
@@ -1740,7 +1743,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" s="1">
         <v>888</v>
@@ -1751,7 +1754,7 @@
       <c r="E10" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="6">
         <v>99999999999</v>
       </c>
     </row>
@@ -1760,7 +1763,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1">
         <v>888</v>
@@ -1771,8 +1774,8 @@
       <c r="E11" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>25</v>
+      <c r="F11" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1780,7 +1783,7 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1">
         <v>888</v>
@@ -1791,8 +1794,8 @@
       <c r="E12" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>27</v>
+      <c r="F12" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1800,7 +1803,7 @@
         <v>16</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1">
         <v>888</v>
@@ -1811,8 +1814,8 @@
       <c r="E13" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>27</v>
+      <c r="F13" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1820,7 +1823,7 @@
         <v>17</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C14" s="1">
         <v>888</v>
@@ -1831,8 +1834,8 @@
       <c r="E14" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>27</v>
+      <c r="F14" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1860,653 +1863,653 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="1">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" s="1">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B9" s="1">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B10" s="1">
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B11" s="1">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B12" s="1">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B13" s="1">
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B14" s="1">
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B15" s="1">
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B16" s="1">
         <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B17" s="1">
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B18" s="1">
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B19" s="1">
         <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B20" s="1">
         <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="1">
         <v>19</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="1">
         <v>20</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B23" s="1">
         <v>21</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B24" s="1">
         <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B25" s="1">
         <v>23</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B26" s="1">
         <v>24</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B27" s="1">
         <v>25</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B28" s="1">
         <v>26</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B29" s="1">
         <v>27</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B30" s="1">
         <v>28</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B31" s="1">
         <v>29</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B32" s="1">
         <v>30</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B33" s="1">
         <v>31</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B34" s="1">
         <v>32</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B35" s="1">
         <v>33</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B36" s="1">
         <v>34</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B37" s="1">
         <v>35</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B38" s="1">
         <v>36</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B39" s="1">
         <v>37</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B40" s="1">
         <v>38</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B41" s="1">
         <v>39</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B42" s="1">
         <v>40</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B43" s="1">
         <v>41</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B44" s="1">
         <v>42</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B45" s="1">
         <v>43</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B46" s="1">
         <v>44</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B47" s="1">
         <v>45</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B48" s="1">
         <v>46</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B49" s="1">
         <v>47</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B50" s="1">
         <v>48</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B51" s="1">
         <v>49</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B52" s="1">
         <v>50</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B53" s="1">
         <v>51</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B54" s="1">
         <v>52</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B55" s="1">
         <v>53</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B56" s="1">
         <v>54</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B57" s="1">
         <v>55</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B58" s="1">
         <v>56</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B59" s="1">
         <v>101</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B60" s="1">
         <v>102</v>
@@ -2515,7 +2518,7 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B61" s="1">
         <v>103</v>
@@ -2524,7 +2527,7 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B62" s="1">
         <v>104</v>
@@ -2533,7 +2536,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B63" s="1">
         <v>105</v>
@@ -2542,7 +2545,7 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B64" s="1">
         <v>106</v>
@@ -2551,7 +2554,7 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B65" s="1">
         <v>107</v>
@@ -2560,7 +2563,7 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B66" s="1">
         <v>108</v>
@@ -2569,7 +2572,7 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B67" s="1">
         <v>109</v>
@@ -2578,35 +2581,35 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B69" s="1">
         <v>201</v>
       </c>
       <c r="C69" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B70" s="1">
         <v>202</v>
       </c>
       <c r="C70" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="72" ht="15" spans="1:3">
       <c r="A72" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B72" s="1">
         <v>888</v>
       </c>
-      <c r="C72" s="5" t="s">
-        <v>161</v>
+      <c r="C72" s="4" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2632,77 +2635,77 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D2" s="4"/>
+        <v>164</v>
+      </c>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B6" s="1">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B7" s="1">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(parser): 适配 protobuf v2 反射接口
</commit_message>
<xml_diff>
--- a/assets/xls/物品.xlsx
+++ b/assets/xls/物品.xlsx
@@ -59,7 +59,7 @@
     <t>i18n</t>
   </si>
   <si>
-    <t>int32</t>
+    <t>ItemType</t>
   </si>
   <si>
     <t>bool</t>
@@ -1579,7 +1579,7 @@
     <col min="1" max="1" width="15.375" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.375" style="1" customWidth="1"/>
     <col min="3" max="3" width="10.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.875" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.25" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.875" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="1"/>
@@ -1616,7 +1616,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>9</v>
@@ -1672,12 +1672,8 @@
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1">
-        <v>1</v>
-      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="6">
         <v>10</v>
@@ -1824,7 +1820,7 @@
         <v>888</v>
       </c>
       <c r="D13" s="1">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1" t="b">
         <v>1</v>
@@ -1844,7 +1840,7 @@
         <v>888</v>
       </c>
       <c r="D14" s="1">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1" t="b">
         <v>1</v>

</xml_diff>